<commit_message>
test(fixtures): hold common names at token weight in late files
Both late-known files now carry every common security at a 1-2 bp token weight, so leaking either into the 2026-11-02 answer moves the SYNA/SYNB overlap by 0.2474 instead of 0.006-0.028. expected_overlap.json is unchanged.
</commit_message>
<xml_diff>
--- a/tests/fixtures/raw_synthetic/synthetic/SYNB/2026-11-02/20261103T150000Z.xlsx
+++ b/tests/fixtures/raw_synthetic/synthetic/SYNB/2026-11-02/20261103T150000Z.xlsx
@@ -502,19 +502,15 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Fairhaven Financial Group</t>
+          <t>Doverdale Textiles Ltd.</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>FHV</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>CA600005AA02</t>
-        </is>
-      </c>
+          <t>DVR</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr"/>
       <c r="D6" t="inlineStr"/>
       <c r="E6" t="inlineStr">
         <is>
@@ -523,7 +519,7 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Utilities</t>
+          <t>Health Care</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
@@ -537,125 +533,125 @@
         </is>
       </c>
       <c r="I6" t="n">
-        <v>0.0917</v>
+        <v>0.07240000000000001</v>
       </c>
       <c r="J6" t="n">
-        <v>9967</v>
+        <v>6582</v>
       </c>
       <c r="K6" t="n">
-        <v>458500</v>
+        <v>362000</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Doverdale Textiles Ltd.</t>
+          <t>Granite Peak Resources</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>DVR</t>
+          <t>GRP</t>
         </is>
       </c>
       <c r="C7" t="inlineStr"/>
-      <c r="D7" t="inlineStr"/>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>200030BA1</t>
+        </is>
+      </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>XTSE</t>
+          <t>XNYS</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Health Care</t>
+          <t>Materials</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>CA</t>
+          <t>US</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>CAD</t>
+          <t>USD</t>
         </is>
       </c>
       <c r="I7" t="n">
-        <v>0.07240000000000001</v>
+        <v>0.0713</v>
       </c>
       <c r="J7" t="n">
-        <v>6582</v>
+        <v>5243</v>
       </c>
       <c r="K7" t="n">
-        <v>362000</v>
+        <v>356500</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Granite Peak Resources</t>
+          <t>Brighton Paper Corp.</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>GRP</t>
+          <t>BRP</t>
         </is>
       </c>
       <c r="C8" t="inlineStr"/>
       <c r="D8" t="inlineStr">
         <is>
-          <t>200030BA1</t>
+          <t>600025AA8</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>XNYS</t>
+          <t>XTSE</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Materials</t>
+          <t>Utilities</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>CA</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>USD</t>
+          <t>CAD</t>
         </is>
       </c>
       <c r="I8" t="n">
-        <v>0.0713</v>
+        <v>0.0624</v>
       </c>
       <c r="J8" t="n">
-        <v>5243</v>
+        <v>10759</v>
       </c>
       <c r="K8" t="n">
-        <v>356500</v>
+        <v>312000</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Glenora Utilities Inc.</t>
+          <t>Maple Ridge Systems Corp.</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>GLO</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>CA600006AA84</t>
-        </is>
-      </c>
+          <t>MAPL</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr"/>
       <c r="D9" t="inlineStr"/>
       <c r="E9" t="inlineStr">
         <is>
-          <t>XTSE</t>
+          <t>XNYS</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
@@ -665,39 +661,39 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>CA</t>
+          <t>US</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>CAD</t>
+          <t>USD</t>
         </is>
       </c>
       <c r="I9" t="n">
-        <v>0.0704</v>
+        <v>0.058</v>
       </c>
       <c r="J9" t="n">
-        <v>5966</v>
+        <v>2339</v>
       </c>
       <c r="K9" t="n">
-        <v>352000</v>
+        <v>290000</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Ironbridge Steel Inc.</t>
+          <t>Westmount Power Corp.</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>IRO</t>
+          <t>WST</t>
         </is>
       </c>
       <c r="C10" t="inlineStr"/>
       <c r="D10" t="inlineStr">
         <is>
-          <t>600008AA4</t>
+          <t>600022AA5</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -707,7 +703,7 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Real Estate</t>
+          <t>Financials</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
@@ -721,118 +717,122 @@
         </is>
       </c>
       <c r="I10" t="n">
-        <v>0.0694</v>
+        <v>0.0548</v>
       </c>
       <c r="J10" t="n">
-        <v>4819</v>
+        <v>1827</v>
       </c>
       <c r="K10" t="n">
-        <v>347000</v>
+        <v>274000</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Brighton Paper Corp.</t>
+          <t>Highwater Marine Corp.</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>BRP</t>
+          <t>HWX</t>
         </is>
       </c>
       <c r="C11" t="inlineStr"/>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>600025AA8</t>
-        </is>
-      </c>
+      <c r="D11" t="inlineStr"/>
       <c r="E11" t="inlineStr">
         <is>
-          <t>XTSE</t>
+          <t>XNYS</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Utilities</t>
+          <t>Energy</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>CA</t>
+          <t>US</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>CAD</t>
+          <t>USD</t>
         </is>
       </c>
       <c r="I11" t="n">
-        <v>0.0624</v>
+        <v>0.0526</v>
       </c>
       <c r="J11" t="n">
-        <v>10759</v>
+        <v>3247</v>
       </c>
       <c r="K11" t="n">
-        <v>312000</v>
+        <v>263000</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Elmsworth Capital Corp.</t>
+          <t>Yarrow Biotech Inc.</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>ELM</t>
+          <t>YAR</t>
         </is>
       </c>
       <c r="C12" t="inlineStr"/>
-      <c r="D12" t="inlineStr"/>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>600023AA3</t>
+        </is>
+      </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>XNYS</t>
+          <t>XTSE</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Real Estate</t>
+          <t>Industrials</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>CA</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>USD</t>
+          <t>CAD</t>
         </is>
       </c>
       <c r="I12" t="n">
-        <v>0.0624</v>
+        <v>0.0509</v>
       </c>
       <c r="J12" t="n">
-        <v>3184</v>
+        <v>1561</v>
       </c>
       <c r="K12" t="n">
-        <v>312000</v>
+        <v>254500</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Foxglove Networks Inc.</t>
+          <t>Ironwood Devices Inc.</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>FXN</t>
+          <t>IRW</t>
         </is>
       </c>
       <c r="C13" t="inlineStr"/>
-      <c r="D13" t="inlineStr"/>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>200032BA7</t>
+        </is>
+      </c>
       <c r="E13" t="inlineStr">
         <is>
           <t>XNYS</t>
@@ -840,7 +840,7 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Communication Services</t>
+          <t>Financials</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
@@ -854,75 +854,71 @@
         </is>
       </c>
       <c r="I13" t="n">
-        <v>0.0591</v>
+        <v>0.0407</v>
       </c>
       <c r="J13" t="n">
-        <v>2662</v>
+        <v>2165</v>
       </c>
       <c r="K13" t="n">
-        <v>295500</v>
+        <v>203500</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Maple Ridge Systems Corp.</t>
+          <t>Aldergrove Metals Ltd.</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>MAPL</t>
+          <t>ALD</t>
         </is>
       </c>
       <c r="C14" t="inlineStr"/>
       <c r="D14" t="inlineStr"/>
       <c r="E14" t="inlineStr">
         <is>
-          <t>XNYS</t>
+          <t>XTSE</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>Information Technology</t>
+          <t>Consumer Staples</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>CA</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>USD</t>
+          <t>CAD</t>
         </is>
       </c>
       <c r="I14" t="n">
-        <v>0.058</v>
+        <v>0.0396</v>
       </c>
       <c r="J14" t="n">
-        <v>2339</v>
+        <v>1125</v>
       </c>
       <c r="K14" t="n">
-        <v>290000</v>
+        <v>198000</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Westmount Power Corp.</t>
+          <t>Cardinal Freight Ltd.</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>WST</t>
+          <t>CFR</t>
         </is>
       </c>
       <c r="C15" t="inlineStr"/>
-      <c r="D15" t="inlineStr">
-        <is>
-          <t>600022AA5</t>
-        </is>
-      </c>
+      <c r="D15" t="inlineStr"/>
       <c r="E15" t="inlineStr">
         <is>
           <t>XTSE</t>
@@ -930,7 +926,7 @@
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>Financials</t>
+          <t>Information Technology</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
@@ -944,31 +940,35 @@
         </is>
       </c>
       <c r="I15" t="n">
-        <v>0.0548</v>
+        <v>0.0309</v>
       </c>
       <c r="J15" t="n">
-        <v>1827</v>
+        <v>3679</v>
       </c>
       <c r="K15" t="n">
-        <v>274000</v>
+        <v>154500</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Highwater Marine Corp.</t>
+          <t>Vermilion Distillers Corp.</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>HWX</t>
+          <t>VRM</t>
         </is>
       </c>
       <c r="C16" t="inlineStr"/>
-      <c r="D16" t="inlineStr"/>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>600021AA7</t>
+        </is>
+      </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>XNYS</t>
+          <t>XTSE</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
@@ -978,39 +978,39 @@
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>CA</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>USD</t>
+          <t>CAD</t>
         </is>
       </c>
       <c r="I16" t="n">
-        <v>0.0526</v>
+        <v>0.0126</v>
       </c>
       <c r="J16" t="n">
-        <v>3247</v>
+        <v>460</v>
       </c>
       <c r="K16" t="n">
-        <v>263000</v>
+        <v>63000</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Yarrow Biotech Inc.</t>
+          <t>Kestrel Aerospace Inc.</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>YAR</t>
+          <t>KES</t>
         </is>
       </c>
       <c r="C17" t="inlineStr"/>
       <c r="D17" t="inlineStr">
         <is>
-          <t>600023AA3</t>
+          <t>600010AA0</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
@@ -1020,7 +1020,7 @@
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>Industrials</t>
+          <t>Materials</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
@@ -1034,29 +1034,29 @@
         </is>
       </c>
       <c r="I17" t="n">
-        <v>0.0509</v>
+        <v>0.0002</v>
       </c>
       <c r="J17" t="n">
-        <v>1561</v>
+        <v>12</v>
       </c>
       <c r="K17" t="n">
-        <v>254500</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Cedarline Energy Corp.</t>
+          <t>Northwind Materials Inc.</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>CDL</t>
+          <t>NWM</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>CA600002AA70</t>
+          <t>CA600000AA15</t>
         </is>
       </c>
       <c r="D18" t="inlineStr"/>
@@ -1067,7 +1067,7 @@
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>Financials</t>
+          <t>Materials</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
@@ -1081,35 +1081,35 @@
         </is>
       </c>
       <c r="I18" t="n">
-        <v>0.05</v>
+        <v>0.0002</v>
       </c>
       <c r="J18" t="n">
-        <v>7576</v>
+        <v>50</v>
       </c>
       <c r="K18" t="n">
-        <v>250000</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Ironwood Devices Inc.</t>
+          <t>Cedarline Energy Corp.</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>IRW</t>
-        </is>
-      </c>
-      <c r="C19" t="inlineStr"/>
-      <c r="D19" t="inlineStr">
-        <is>
-          <t>200032BA7</t>
-        </is>
-      </c>
+          <t>CDL</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>CA600002AA70</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr"/>
       <c r="E19" t="inlineStr">
         <is>
-          <t>XNYS</t>
+          <t>XTSE</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
@@ -1119,84 +1119,84 @@
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>CA</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>USD</t>
+          <t>CAD</t>
         </is>
       </c>
       <c r="I19" t="n">
-        <v>0.0407</v>
+        <v>0.0001</v>
       </c>
       <c r="J19" t="n">
-        <v>2165</v>
+        <v>15</v>
       </c>
       <c r="K19" t="n">
-        <v>203500</v>
+        <v>500</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Aldergrove Metals Ltd.</t>
+          <t>Elmsworth Capital Corp.</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>ALD</t>
+          <t>ELM</t>
         </is>
       </c>
       <c r="C20" t="inlineStr"/>
       <c r="D20" t="inlineStr"/>
       <c r="E20" t="inlineStr">
         <is>
-          <t>XTSE</t>
+          <t>XNYS</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>Consumer Staples</t>
+          <t>Real Estate</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>CA</t>
+          <t>US</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>CAD</t>
+          <t>USD</t>
         </is>
       </c>
       <c r="I20" t="n">
-        <v>0.0396</v>
+        <v>0.0001</v>
       </c>
       <c r="J20" t="n">
-        <v>1125</v>
+        <v>5</v>
       </c>
       <c r="K20" t="n">
-        <v>198000</v>
+        <v>500</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Kestrel Aerospace Inc.</t>
+          <t>Fairhaven Financial Group</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>KES</t>
-        </is>
-      </c>
-      <c r="C21" t="inlineStr"/>
-      <c r="D21" t="inlineStr">
-        <is>
-          <t>600010AA0</t>
-        </is>
-      </c>
+          <t>FHV</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>CA600005AA02</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr"/>
       <c r="E21" t="inlineStr">
         <is>
           <t>XTSE</t>
@@ -1204,7 +1204,7 @@
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>Materials</t>
+          <t>Utilities</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
@@ -1218,75 +1218,75 @@
         </is>
       </c>
       <c r="I21" t="n">
-        <v>0.037</v>
+        <v>0.0001</v>
       </c>
       <c r="J21" t="n">
-        <v>2176</v>
+        <v>11</v>
       </c>
       <c r="K21" t="n">
-        <v>185000</v>
+        <v>500</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Cardinal Freight Ltd.</t>
+          <t>Foxglove Networks Inc.</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>CFR</t>
+          <t>FXN</t>
         </is>
       </c>
       <c r="C22" t="inlineStr"/>
       <c r="D22" t="inlineStr"/>
       <c r="E22" t="inlineStr">
         <is>
-          <t>XTSE</t>
+          <t>XNYS</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>Information Technology</t>
+          <t>Communication Services</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>CA</t>
+          <t>US</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>CAD</t>
+          <t>USD</t>
         </is>
       </c>
       <c r="I22" t="n">
-        <v>0.0309</v>
+        <v>0.0001</v>
       </c>
       <c r="J22" t="n">
-        <v>3679</v>
+        <v>5</v>
       </c>
       <c r="K22" t="n">
-        <v>154500</v>
+        <v>500</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Vermilion Distillers Corp.</t>
+          <t>Glenora Utilities Inc.</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>VRM</t>
-        </is>
-      </c>
-      <c r="C23" t="inlineStr"/>
-      <c r="D23" t="inlineStr">
-        <is>
-          <t>600021AA7</t>
-        </is>
-      </c>
+          <t>GLO</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>CA600006AA84</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr"/>
       <c r="E23" t="inlineStr">
         <is>
           <t>XTSE</t>
@@ -1294,7 +1294,7 @@
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>Energy</t>
+          <t>Information Technology</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
@@ -1308,32 +1308,32 @@
         </is>
       </c>
       <c r="I23" t="n">
-        <v>0.0126</v>
+        <v>0.0001</v>
       </c>
       <c r="J23" t="n">
-        <v>460</v>
+        <v>8</v>
       </c>
       <c r="K23" t="n">
-        <v>63000</v>
+        <v>500</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Northwind Materials Inc.</t>
+          <t>Ironbridge Steel Inc.</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>NWM</t>
-        </is>
-      </c>
-      <c r="C24" t="inlineStr">
-        <is>
-          <t>CA600000AA15</t>
-        </is>
-      </c>
-      <c r="D24" t="inlineStr"/>
+          <t>IRO</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr"/>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>600008AA4</t>
+        </is>
+      </c>
       <c r="E24" t="inlineStr">
         <is>
           <t>XTSE</t>
@@ -1341,7 +1341,7 @@
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>Materials</t>
+          <t>Real Estate</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
@@ -1355,13 +1355,13 @@
         </is>
       </c>
       <c r="I24" t="n">
-        <v>0.004</v>
+        <v>0.0001</v>
       </c>
       <c r="J24" t="n">
-        <v>1000</v>
+        <v>7</v>
       </c>
       <c r="K24" t="n">
-        <v>20000</v>
+        <v>500</v>
       </c>
     </row>
     <row r="25">
@@ -1386,13 +1386,13 @@
         </is>
       </c>
       <c r="I25" t="n">
-        <v>0.0098</v>
+        <v>0.4528</v>
       </c>
       <c r="J25" t="n">
         <v>0</v>
       </c>
       <c r="K25" t="n">
-        <v>49000</v>
+        <v>2264000</v>
       </c>
     </row>
   </sheetData>

</xml_diff>